<commit_message>
Added revised test data for top model Moran's I test. I still need to extract residuals for the model average and the individual mixed models in order to test for spatial autocorrelation in them.
</commit_message>
<xml_diff>
--- a/Data/moran_test_data.xlsx
+++ b/Data/moran_test_data.xlsx
@@ -408,7 +408,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.1150251122526957</v>
+        <v>-0.05587411029387779</v>
       </c>
       <c r="C2">
         <v>36.8253</v>
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>-0.03250727312865076</v>
+        <v>0.08593813951782803</v>
       </c>
       <c r="C3">
         <v>36.9299</v>
@@ -486,7 +486,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.1588349496461766</v>
+        <v>0.2227288630892927</v>
       </c>
       <c r="C4">
         <v>36.9356</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.03453583759517694</v>
+        <v>0.01358533081888592</v>
       </c>
       <c r="C5">
         <v>36.9568</v>
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>-0.3168678076158216</v>
+        <v>-0.335474757799711</v>
       </c>
       <c r="C6">
         <v>36.7769</v>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>0.1407700345586296</v>
+        <v>0.1732761547309193</v>
       </c>
       <c r="C7">
         <v>36.8612</v>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>-0.05955686479834132</v>
+        <v>-0.05186124176639728</v>
       </c>
       <c r="C8">
         <v>36.8612</v>
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>-0.3116064048721075</v>
+        <v>-0.3119404217146562</v>
       </c>
       <c r="C9">
         <v>36.7816</v>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>-0.1078754233572941</v>
+        <v>-0.1217496009610147</v>
       </c>
       <c r="C10">
         <v>36.9235</v>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>0.0923907687123619</v>
+        <v>0.07440474694593291</v>
       </c>
       <c r="C11">
         <v>36.9234</v>
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>-0.1719418293967707</v>
+        <v>-0.1810869720816495</v>
       </c>
       <c r="C12">
         <v>36.8263</v>
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>0.08004407620737797</v>
+        <v>0.03027888171820692</v>
       </c>
       <c r="C13">
         <v>36.8269</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>0.5066761112295723</v>
+        <v>0.259163687574455</v>
       </c>
       <c r="C14">
         <v>36.814</v>
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>-0.2625860381262826</v>
+        <v>-0.2510676122166792</v>
       </c>
       <c r="C15">
         <v>36.8206</v>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>-0.1655373606738981</v>
+        <v>-0.1671667130655452</v>
       </c>
       <c r="C16">
         <v>36.8393</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>-0.2286856989482424</v>
+        <v>-0.2348345526101461</v>
       </c>
       <c r="C17">
         <v>36.9708</v>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>-0.3540239890036772</v>
+        <v>-0.3670547718310334</v>
       </c>
       <c r="C18">
         <v>36.9711</v>
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="B19">
-        <v>0.01675864955134132</v>
+        <v>-0.01134138359565536</v>
       </c>
       <c r="C19">
         <v>36.9704</v>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>0.1862435075412031</v>
+        <v>0.2535635997991028</v>
       </c>
       <c r="C20">
         <v>36.7849</v>
@@ -1149,7 +1149,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>-0.1347348432540536</v>
+        <v>-0.166014341339715</v>
       </c>
       <c r="C21">
         <v>36.7911</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>-0.1535279853269433</v>
+        <v>-0.1829289837521282</v>
       </c>
       <c r="C22">
         <v>36.8576</v>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>0.176684212067499</v>
+        <v>0.2100836782966924</v>
       </c>
       <c r="C23">
         <v>36.8586</v>
@@ -1266,7 +1266,7 @@
         </is>
       </c>
       <c r="B24">
-        <v>0.2267990114884146</v>
+        <v>0.1976323054283769</v>
       </c>
       <c r="C24">
         <v>36.8597</v>
@@ -1305,7 +1305,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>0.07357260811561919</v>
+        <v>0.1185213235889502</v>
       </c>
       <c r="C25">
         <v>36.8584</v>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="B26">
-        <v>0.1129717470323548</v>
+        <v>0.1472475667305279</v>
       </c>
       <c r="C26">
         <v>36.8595</v>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.1767136858881932</v>
+        <v>0.2126604176771378</v>
       </c>
       <c r="C27">
         <v>36.9213</v>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>0.253110877820868</v>
+        <v>0.2842435049381404</v>
       </c>
       <c r="C28">
         <v>36.9671</v>
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>0.02907527963102874</v>
+        <v>0.01106585275686772</v>
       </c>
       <c r="C29">
         <v>36.9586</v>
@@ -1500,7 +1500,7 @@
         </is>
       </c>
       <c r="B30">
-        <v>0.06538193893797795</v>
+        <v>0.09075974644797941</v>
       </c>
       <c r="C30">
         <v>36.9554</v>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="B31">
-        <v>0.2321374994590088</v>
+        <v>0.2388038472606171</v>
       </c>
       <c r="C31">
         <v>36.959</v>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="B32">
-        <v>-0.4281232479447008</v>
+        <v>-0.3651501075106304</v>
       </c>
       <c r="C32">
         <v>36.9802</v>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="B33">
-        <v>-0.05441164797603704</v>
+        <v>-0.09635151454115076</v>
       </c>
       <c r="C33">
         <v>36.7757</v>
@@ -1656,7 +1656,7 @@
         </is>
       </c>
       <c r="B34">
-        <v>-0.004125247269532932</v>
+        <v>-0.03000629982136123</v>
       </c>
       <c r="C34">
         <v>36.9555</v>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="B35">
-        <v>-0.1100468542714466</v>
+        <v>-0.09093981026592579</v>
       </c>
       <c r="C35">
         <v>36.8243</v>
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="B36">
-        <v>-0.2091723501596162</v>
+        <v>-0.1510974044659294</v>
       </c>
       <c r="C36">
         <v>36.9818</v>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="B37">
-        <v>-0.02649197426905364</v>
+        <v>-0.05113044139086415</v>
       </c>
       <c r="C37">
         <v>36.8205</v>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="B38">
-        <v>0.1301671927763302</v>
+        <v>0.07197498527146326</v>
       </c>
       <c r="C38">
         <v>36.9731</v>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B39">
-        <v>-0.215182492663374</v>
+        <v>-0.2305517084666777</v>
       </c>
       <c r="C39">
         <v>36.8167</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="B40">
-        <v>0.4114879393690004</v>
+        <v>0.4447457998792453</v>
       </c>
       <c r="C40">
         <v>36.964</v>
@@ -1929,7 +1929,7 @@
         </is>
       </c>
       <c r="B41">
-        <v>-0.03216140962409952</v>
+        <v>-0.06042876124183338</v>
       </c>
       <c r="C41">
         <v>36.8324</v>

</xml_diff>